<commit_message>
Plantilla de personas: cargo libre, sin columnas de admin, foto ni notas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L8QtHgV8HSYntBJ1ppQiSV
</commit_message>
<xml_diff>
--- a/borradores/rabbit-personas.xlsx
+++ b/borradores/rabbit-personas.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K101"/>
+  <dimension ref="A1:H101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -454,12 +454,9 @@
     <col width="34" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="30" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -490,32 +487,17 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Rol en Rabbit *</t>
+          <t>Cargo *</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>¿Administra Personas?</t>
+          <t>Fecha de cumpleaños</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Fecha de cumpleaños</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
           <t>Celular (WhatsApp)</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Foto (nombre del archivo)</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Notas</t>
         </is>
       </c>
     </row>
@@ -552,27 +534,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>15/03</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>15/03</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
           <t>999 999 999</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>hilary.jpg</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>Ejemplo: bórrala y escribe los datos reales</t>
         </is>
       </c>
     </row>
@@ -585,9 +552,6 @@
       <c r="F3" s="3" t="n"/>
       <c r="G3" s="3" t="n"/>
       <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="n"/>
-      <c r="K3" s="3" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="n"/>
@@ -598,9 +562,6 @@
       <c r="F4" s="3" t="n"/>
       <c r="G4" s="3" t="n"/>
       <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="3" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n"/>
@@ -611,9 +572,6 @@
       <c r="F5" s="3" t="n"/>
       <c r="G5" s="3" t="n"/>
       <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="n"/>
-      <c r="K5" s="3" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n"/>
@@ -624,9 +582,6 @@
       <c r="F6" s="3" t="n"/>
       <c r="G6" s="3" t="n"/>
       <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="3" t="n"/>
-      <c r="K6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n"/>
@@ -637,9 +592,6 @@
       <c r="F7" s="3" t="n"/>
       <c r="G7" s="3" t="n"/>
       <c r="H7" s="3" t="n"/>
-      <c r="I7" s="3" t="n"/>
-      <c r="J7" s="3" t="n"/>
-      <c r="K7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n"/>
@@ -650,9 +602,6 @@
       <c r="F8" s="3" t="n"/>
       <c r="G8" s="3" t="n"/>
       <c r="H8" s="3" t="n"/>
-      <c r="I8" s="3" t="n"/>
-      <c r="J8" s="3" t="n"/>
-      <c r="K8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n"/>
@@ -663,9 +612,6 @@
       <c r="F9" s="3" t="n"/>
       <c r="G9" s="3" t="n"/>
       <c r="H9" s="3" t="n"/>
-      <c r="I9" s="3" t="n"/>
-      <c r="J9" s="3" t="n"/>
-      <c r="K9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n"/>
@@ -676,9 +622,6 @@
       <c r="F10" s="3" t="n"/>
       <c r="G10" s="3" t="n"/>
       <c r="H10" s="3" t="n"/>
-      <c r="I10" s="3" t="n"/>
-      <c r="J10" s="3" t="n"/>
-      <c r="K10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n"/>
@@ -689,9 +632,6 @@
       <c r="F11" s="3" t="n"/>
       <c r="G11" s="3" t="n"/>
       <c r="H11" s="3" t="n"/>
-      <c r="I11" s="3" t="n"/>
-      <c r="J11" s="3" t="n"/>
-      <c r="K11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n"/>
@@ -702,9 +642,6 @@
       <c r="F12" s="3" t="n"/>
       <c r="G12" s="3" t="n"/>
       <c r="H12" s="3" t="n"/>
-      <c r="I12" s="3" t="n"/>
-      <c r="J12" s="3" t="n"/>
-      <c r="K12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n"/>
@@ -715,9 +652,6 @@
       <c r="F13" s="3" t="n"/>
       <c r="G13" s="3" t="n"/>
       <c r="H13" s="3" t="n"/>
-      <c r="I13" s="3" t="n"/>
-      <c r="J13" s="3" t="n"/>
-      <c r="K13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n"/>
@@ -728,9 +662,6 @@
       <c r="F14" s="3" t="n"/>
       <c r="G14" s="3" t="n"/>
       <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="n"/>
-      <c r="J14" s="3" t="n"/>
-      <c r="K14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n"/>
@@ -741,9 +672,6 @@
       <c r="F15" s="3" t="n"/>
       <c r="G15" s="3" t="n"/>
       <c r="H15" s="3" t="n"/>
-      <c r="I15" s="3" t="n"/>
-      <c r="J15" s="3" t="n"/>
-      <c r="K15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n"/>
@@ -754,9 +682,6 @@
       <c r="F16" s="3" t="n"/>
       <c r="G16" s="3" t="n"/>
       <c r="H16" s="3" t="n"/>
-      <c r="I16" s="3" t="n"/>
-      <c r="J16" s="3" t="n"/>
-      <c r="K16" s="3" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n"/>
@@ -767,9 +692,6 @@
       <c r="F17" s="3" t="n"/>
       <c r="G17" s="3" t="n"/>
       <c r="H17" s="3" t="n"/>
-      <c r="I17" s="3" t="n"/>
-      <c r="J17" s="3" t="n"/>
-      <c r="K17" s="3" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n"/>
@@ -780,9 +702,6 @@
       <c r="F18" s="3" t="n"/>
       <c r="G18" s="3" t="n"/>
       <c r="H18" s="3" t="n"/>
-      <c r="I18" s="3" t="n"/>
-      <c r="J18" s="3" t="n"/>
-      <c r="K18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n"/>
@@ -793,9 +712,6 @@
       <c r="F19" s="3" t="n"/>
       <c r="G19" s="3" t="n"/>
       <c r="H19" s="3" t="n"/>
-      <c r="I19" s="3" t="n"/>
-      <c r="J19" s="3" t="n"/>
-      <c r="K19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n"/>
@@ -806,9 +722,6 @@
       <c r="F20" s="3" t="n"/>
       <c r="G20" s="3" t="n"/>
       <c r="H20" s="3" t="n"/>
-      <c r="I20" s="3" t="n"/>
-      <c r="J20" s="3" t="n"/>
-      <c r="K20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n"/>
@@ -819,9 +732,6 @@
       <c r="F21" s="3" t="n"/>
       <c r="G21" s="3" t="n"/>
       <c r="H21" s="3" t="n"/>
-      <c r="I21" s="3" t="n"/>
-      <c r="J21" s="3" t="n"/>
-      <c r="K21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n"/>
@@ -832,9 +742,6 @@
       <c r="F22" s="3" t="n"/>
       <c r="G22" s="3" t="n"/>
       <c r="H22" s="3" t="n"/>
-      <c r="I22" s="3" t="n"/>
-      <c r="J22" s="3" t="n"/>
-      <c r="K22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n"/>
@@ -845,9 +752,6 @@
       <c r="F23" s="3" t="n"/>
       <c r="G23" s="3" t="n"/>
       <c r="H23" s="3" t="n"/>
-      <c r="I23" s="3" t="n"/>
-      <c r="J23" s="3" t="n"/>
-      <c r="K23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n"/>
@@ -858,9 +762,6 @@
       <c r="F24" s="3" t="n"/>
       <c r="G24" s="3" t="n"/>
       <c r="H24" s="3" t="n"/>
-      <c r="I24" s="3" t="n"/>
-      <c r="J24" s="3" t="n"/>
-      <c r="K24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n"/>
@@ -871,9 +772,6 @@
       <c r="F25" s="3" t="n"/>
       <c r="G25" s="3" t="n"/>
       <c r="H25" s="3" t="n"/>
-      <c r="I25" s="3" t="n"/>
-      <c r="J25" s="3" t="n"/>
-      <c r="K25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n"/>
@@ -884,9 +782,6 @@
       <c r="F26" s="3" t="n"/>
       <c r="G26" s="3" t="n"/>
       <c r="H26" s="3" t="n"/>
-      <c r="I26" s="3" t="n"/>
-      <c r="J26" s="3" t="n"/>
-      <c r="K26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n"/>
@@ -897,9 +792,6 @@
       <c r="F27" s="3" t="n"/>
       <c r="G27" s="3" t="n"/>
       <c r="H27" s="3" t="n"/>
-      <c r="I27" s="3" t="n"/>
-      <c r="J27" s="3" t="n"/>
-      <c r="K27" s="3" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n"/>
@@ -910,9 +802,6 @@
       <c r="F28" s="3" t="n"/>
       <c r="G28" s="3" t="n"/>
       <c r="H28" s="3" t="n"/>
-      <c r="I28" s="3" t="n"/>
-      <c r="J28" s="3" t="n"/>
-      <c r="K28" s="3" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n"/>
@@ -923,9 +812,6 @@
       <c r="F29" s="3" t="n"/>
       <c r="G29" s="3" t="n"/>
       <c r="H29" s="3" t="n"/>
-      <c r="I29" s="3" t="n"/>
-      <c r="J29" s="3" t="n"/>
-      <c r="K29" s="3" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n"/>
@@ -936,9 +822,6 @@
       <c r="F30" s="3" t="n"/>
       <c r="G30" s="3" t="n"/>
       <c r="H30" s="3" t="n"/>
-      <c r="I30" s="3" t="n"/>
-      <c r="J30" s="3" t="n"/>
-      <c r="K30" s="3" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n"/>
@@ -949,9 +832,6 @@
       <c r="F31" s="3" t="n"/>
       <c r="G31" s="3" t="n"/>
       <c r="H31" s="3" t="n"/>
-      <c r="I31" s="3" t="n"/>
-      <c r="J31" s="3" t="n"/>
-      <c r="K31" s="3" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n"/>
@@ -962,9 +842,6 @@
       <c r="F32" s="3" t="n"/>
       <c r="G32" s="3" t="n"/>
       <c r="H32" s="3" t="n"/>
-      <c r="I32" s="3" t="n"/>
-      <c r="J32" s="3" t="n"/>
-      <c r="K32" s="3" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n"/>
@@ -975,9 +852,6 @@
       <c r="F33" s="3" t="n"/>
       <c r="G33" s="3" t="n"/>
       <c r="H33" s="3" t="n"/>
-      <c r="I33" s="3" t="n"/>
-      <c r="J33" s="3" t="n"/>
-      <c r="K33" s="3" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n"/>
@@ -988,9 +862,6 @@
       <c r="F34" s="3" t="n"/>
       <c r="G34" s="3" t="n"/>
       <c r="H34" s="3" t="n"/>
-      <c r="I34" s="3" t="n"/>
-      <c r="J34" s="3" t="n"/>
-      <c r="K34" s="3" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n"/>
@@ -1001,9 +872,6 @@
       <c r="F35" s="3" t="n"/>
       <c r="G35" s="3" t="n"/>
       <c r="H35" s="3" t="n"/>
-      <c r="I35" s="3" t="n"/>
-      <c r="J35" s="3" t="n"/>
-      <c r="K35" s="3" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="3" t="n"/>
@@ -1014,9 +882,6 @@
       <c r="F36" s="3" t="n"/>
       <c r="G36" s="3" t="n"/>
       <c r="H36" s="3" t="n"/>
-      <c r="I36" s="3" t="n"/>
-      <c r="J36" s="3" t="n"/>
-      <c r="K36" s="3" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="3" t="n"/>
@@ -1027,9 +892,6 @@
       <c r="F37" s="3" t="n"/>
       <c r="G37" s="3" t="n"/>
       <c r="H37" s="3" t="n"/>
-      <c r="I37" s="3" t="n"/>
-      <c r="J37" s="3" t="n"/>
-      <c r="K37" s="3" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="n"/>
@@ -1040,9 +902,6 @@
       <c r="F38" s="3" t="n"/>
       <c r="G38" s="3" t="n"/>
       <c r="H38" s="3" t="n"/>
-      <c r="I38" s="3" t="n"/>
-      <c r="J38" s="3" t="n"/>
-      <c r="K38" s="3" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="3" t="n"/>
@@ -1053,9 +912,6 @@
       <c r="F39" s="3" t="n"/>
       <c r="G39" s="3" t="n"/>
       <c r="H39" s="3" t="n"/>
-      <c r="I39" s="3" t="n"/>
-      <c r="J39" s="3" t="n"/>
-      <c r="K39" s="3" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="n"/>
@@ -1066,9 +922,6 @@
       <c r="F40" s="3" t="n"/>
       <c r="G40" s="3" t="n"/>
       <c r="H40" s="3" t="n"/>
-      <c r="I40" s="3" t="n"/>
-      <c r="J40" s="3" t="n"/>
-      <c r="K40" s="3" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="n"/>
@@ -1079,9 +932,6 @@
       <c r="F41" s="3" t="n"/>
       <c r="G41" s="3" t="n"/>
       <c r="H41" s="3" t="n"/>
-      <c r="I41" s="3" t="n"/>
-      <c r="J41" s="3" t="n"/>
-      <c r="K41" s="3" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="n"/>
@@ -1092,9 +942,6 @@
       <c r="F42" s="3" t="n"/>
       <c r="G42" s="3" t="n"/>
       <c r="H42" s="3" t="n"/>
-      <c r="I42" s="3" t="n"/>
-      <c r="J42" s="3" t="n"/>
-      <c r="K42" s="3" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="3" t="n"/>
@@ -1105,9 +952,6 @@
       <c r="F43" s="3" t="n"/>
       <c r="G43" s="3" t="n"/>
       <c r="H43" s="3" t="n"/>
-      <c r="I43" s="3" t="n"/>
-      <c r="J43" s="3" t="n"/>
-      <c r="K43" s="3" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="3" t="n"/>
@@ -1118,9 +962,6 @@
       <c r="F44" s="3" t="n"/>
       <c r="G44" s="3" t="n"/>
       <c r="H44" s="3" t="n"/>
-      <c r="I44" s="3" t="n"/>
-      <c r="J44" s="3" t="n"/>
-      <c r="K44" s="3" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="3" t="n"/>
@@ -1131,9 +972,6 @@
       <c r="F45" s="3" t="n"/>
       <c r="G45" s="3" t="n"/>
       <c r="H45" s="3" t="n"/>
-      <c r="I45" s="3" t="n"/>
-      <c r="J45" s="3" t="n"/>
-      <c r="K45" s="3" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="3" t="n"/>
@@ -1144,9 +982,6 @@
       <c r="F46" s="3" t="n"/>
       <c r="G46" s="3" t="n"/>
       <c r="H46" s="3" t="n"/>
-      <c r="I46" s="3" t="n"/>
-      <c r="J46" s="3" t="n"/>
-      <c r="K46" s="3" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="3" t="n"/>
@@ -1157,9 +992,6 @@
       <c r="F47" s="3" t="n"/>
       <c r="G47" s="3" t="n"/>
       <c r="H47" s="3" t="n"/>
-      <c r="I47" s="3" t="n"/>
-      <c r="J47" s="3" t="n"/>
-      <c r="K47" s="3" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n"/>
@@ -1170,9 +1002,6 @@
       <c r="F48" s="3" t="n"/>
       <c r="G48" s="3" t="n"/>
       <c r="H48" s="3" t="n"/>
-      <c r="I48" s="3" t="n"/>
-      <c r="J48" s="3" t="n"/>
-      <c r="K48" s="3" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n"/>
@@ -1183,9 +1012,6 @@
       <c r="F49" s="3" t="n"/>
       <c r="G49" s="3" t="n"/>
       <c r="H49" s="3" t="n"/>
-      <c r="I49" s="3" t="n"/>
-      <c r="J49" s="3" t="n"/>
-      <c r="K49" s="3" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="3" t="n"/>
@@ -1196,9 +1022,6 @@
       <c r="F50" s="3" t="n"/>
       <c r="G50" s="3" t="n"/>
       <c r="H50" s="3" t="n"/>
-      <c r="I50" s="3" t="n"/>
-      <c r="J50" s="3" t="n"/>
-      <c r="K50" s="3" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="3" t="n"/>
@@ -1209,9 +1032,6 @@
       <c r="F51" s="3" t="n"/>
       <c r="G51" s="3" t="n"/>
       <c r="H51" s="3" t="n"/>
-      <c r="I51" s="3" t="n"/>
-      <c r="J51" s="3" t="n"/>
-      <c r="K51" s="3" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="3" t="n"/>
@@ -1222,9 +1042,6 @@
       <c r="F52" s="3" t="n"/>
       <c r="G52" s="3" t="n"/>
       <c r="H52" s="3" t="n"/>
-      <c r="I52" s="3" t="n"/>
-      <c r="J52" s="3" t="n"/>
-      <c r="K52" s="3" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="3" t="n"/>
@@ -1235,9 +1052,6 @@
       <c r="F53" s="3" t="n"/>
       <c r="G53" s="3" t="n"/>
       <c r="H53" s="3" t="n"/>
-      <c r="I53" s="3" t="n"/>
-      <c r="J53" s="3" t="n"/>
-      <c r="K53" s="3" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n"/>
@@ -1248,9 +1062,6 @@
       <c r="F54" s="3" t="n"/>
       <c r="G54" s="3" t="n"/>
       <c r="H54" s="3" t="n"/>
-      <c r="I54" s="3" t="n"/>
-      <c r="J54" s="3" t="n"/>
-      <c r="K54" s="3" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="3" t="n"/>
@@ -1261,9 +1072,6 @@
       <c r="F55" s="3" t="n"/>
       <c r="G55" s="3" t="n"/>
       <c r="H55" s="3" t="n"/>
-      <c r="I55" s="3" t="n"/>
-      <c r="J55" s="3" t="n"/>
-      <c r="K55" s="3" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="3" t="n"/>
@@ -1274,9 +1082,6 @@
       <c r="F56" s="3" t="n"/>
       <c r="G56" s="3" t="n"/>
       <c r="H56" s="3" t="n"/>
-      <c r="I56" s="3" t="n"/>
-      <c r="J56" s="3" t="n"/>
-      <c r="K56" s="3" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="n"/>
@@ -1287,9 +1092,6 @@
       <c r="F57" s="3" t="n"/>
       <c r="G57" s="3" t="n"/>
       <c r="H57" s="3" t="n"/>
-      <c r="I57" s="3" t="n"/>
-      <c r="J57" s="3" t="n"/>
-      <c r="K57" s="3" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="3" t="n"/>
@@ -1300,9 +1102,6 @@
       <c r="F58" s="3" t="n"/>
       <c r="G58" s="3" t="n"/>
       <c r="H58" s="3" t="n"/>
-      <c r="I58" s="3" t="n"/>
-      <c r="J58" s="3" t="n"/>
-      <c r="K58" s="3" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="3" t="n"/>
@@ -1313,9 +1112,6 @@
       <c r="F59" s="3" t="n"/>
       <c r="G59" s="3" t="n"/>
       <c r="H59" s="3" t="n"/>
-      <c r="I59" s="3" t="n"/>
-      <c r="J59" s="3" t="n"/>
-      <c r="K59" s="3" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="3" t="n"/>
@@ -1326,9 +1122,6 @@
       <c r="F60" s="3" t="n"/>
       <c r="G60" s="3" t="n"/>
       <c r="H60" s="3" t="n"/>
-      <c r="I60" s="3" t="n"/>
-      <c r="J60" s="3" t="n"/>
-      <c r="K60" s="3" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="3" t="n"/>
@@ -1339,9 +1132,6 @@
       <c r="F61" s="3" t="n"/>
       <c r="G61" s="3" t="n"/>
       <c r="H61" s="3" t="n"/>
-      <c r="I61" s="3" t="n"/>
-      <c r="J61" s="3" t="n"/>
-      <c r="K61" s="3" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="3" t="n"/>
@@ -1352,9 +1142,6 @@
       <c r="F62" s="3" t="n"/>
       <c r="G62" s="3" t="n"/>
       <c r="H62" s="3" t="n"/>
-      <c r="I62" s="3" t="n"/>
-      <c r="J62" s="3" t="n"/>
-      <c r="K62" s="3" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="3" t="n"/>
@@ -1365,9 +1152,6 @@
       <c r="F63" s="3" t="n"/>
       <c r="G63" s="3" t="n"/>
       <c r="H63" s="3" t="n"/>
-      <c r="I63" s="3" t="n"/>
-      <c r="J63" s="3" t="n"/>
-      <c r="K63" s="3" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="3" t="n"/>
@@ -1378,9 +1162,6 @@
       <c r="F64" s="3" t="n"/>
       <c r="G64" s="3" t="n"/>
       <c r="H64" s="3" t="n"/>
-      <c r="I64" s="3" t="n"/>
-      <c r="J64" s="3" t="n"/>
-      <c r="K64" s="3" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="3" t="n"/>
@@ -1391,9 +1172,6 @@
       <c r="F65" s="3" t="n"/>
       <c r="G65" s="3" t="n"/>
       <c r="H65" s="3" t="n"/>
-      <c r="I65" s="3" t="n"/>
-      <c r="J65" s="3" t="n"/>
-      <c r="K65" s="3" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="3" t="n"/>
@@ -1404,9 +1182,6 @@
       <c r="F66" s="3" t="n"/>
       <c r="G66" s="3" t="n"/>
       <c r="H66" s="3" t="n"/>
-      <c r="I66" s="3" t="n"/>
-      <c r="J66" s="3" t="n"/>
-      <c r="K66" s="3" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="3" t="n"/>
@@ -1417,9 +1192,6 @@
       <c r="F67" s="3" t="n"/>
       <c r="G67" s="3" t="n"/>
       <c r="H67" s="3" t="n"/>
-      <c r="I67" s="3" t="n"/>
-      <c r="J67" s="3" t="n"/>
-      <c r="K67" s="3" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="3" t="n"/>
@@ -1430,9 +1202,6 @@
       <c r="F68" s="3" t="n"/>
       <c r="G68" s="3" t="n"/>
       <c r="H68" s="3" t="n"/>
-      <c r="I68" s="3" t="n"/>
-      <c r="J68" s="3" t="n"/>
-      <c r="K68" s="3" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="3" t="n"/>
@@ -1443,9 +1212,6 @@
       <c r="F69" s="3" t="n"/>
       <c r="G69" s="3" t="n"/>
       <c r="H69" s="3" t="n"/>
-      <c r="I69" s="3" t="n"/>
-      <c r="J69" s="3" t="n"/>
-      <c r="K69" s="3" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="3" t="n"/>
@@ -1456,9 +1222,6 @@
       <c r="F70" s="3" t="n"/>
       <c r="G70" s="3" t="n"/>
       <c r="H70" s="3" t="n"/>
-      <c r="I70" s="3" t="n"/>
-      <c r="J70" s="3" t="n"/>
-      <c r="K70" s="3" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="3" t="n"/>
@@ -1469,9 +1232,6 @@
       <c r="F71" s="3" t="n"/>
       <c r="G71" s="3" t="n"/>
       <c r="H71" s="3" t="n"/>
-      <c r="I71" s="3" t="n"/>
-      <c r="J71" s="3" t="n"/>
-      <c r="K71" s="3" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="3" t="n"/>
@@ -1482,9 +1242,6 @@
       <c r="F72" s="3" t="n"/>
       <c r="G72" s="3" t="n"/>
       <c r="H72" s="3" t="n"/>
-      <c r="I72" s="3" t="n"/>
-      <c r="J72" s="3" t="n"/>
-      <c r="K72" s="3" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="3" t="n"/>
@@ -1495,9 +1252,6 @@
       <c r="F73" s="3" t="n"/>
       <c r="G73" s="3" t="n"/>
       <c r="H73" s="3" t="n"/>
-      <c r="I73" s="3" t="n"/>
-      <c r="J73" s="3" t="n"/>
-      <c r="K73" s="3" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="3" t="n"/>
@@ -1508,9 +1262,6 @@
       <c r="F74" s="3" t="n"/>
       <c r="G74" s="3" t="n"/>
       <c r="H74" s="3" t="n"/>
-      <c r="I74" s="3" t="n"/>
-      <c r="J74" s="3" t="n"/>
-      <c r="K74" s="3" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="3" t="n"/>
@@ -1521,9 +1272,6 @@
       <c r="F75" s="3" t="n"/>
       <c r="G75" s="3" t="n"/>
       <c r="H75" s="3" t="n"/>
-      <c r="I75" s="3" t="n"/>
-      <c r="J75" s="3" t="n"/>
-      <c r="K75" s="3" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="3" t="n"/>
@@ -1534,9 +1282,6 @@
       <c r="F76" s="3" t="n"/>
       <c r="G76" s="3" t="n"/>
       <c r="H76" s="3" t="n"/>
-      <c r="I76" s="3" t="n"/>
-      <c r="J76" s="3" t="n"/>
-      <c r="K76" s="3" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="3" t="n"/>
@@ -1547,9 +1292,6 @@
       <c r="F77" s="3" t="n"/>
       <c r="G77" s="3" t="n"/>
       <c r="H77" s="3" t="n"/>
-      <c r="I77" s="3" t="n"/>
-      <c r="J77" s="3" t="n"/>
-      <c r="K77" s="3" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="3" t="n"/>
@@ -1560,9 +1302,6 @@
       <c r="F78" s="3" t="n"/>
       <c r="G78" s="3" t="n"/>
       <c r="H78" s="3" t="n"/>
-      <c r="I78" s="3" t="n"/>
-      <c r="J78" s="3" t="n"/>
-      <c r="K78" s="3" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="3" t="n"/>
@@ -1573,9 +1312,6 @@
       <c r="F79" s="3" t="n"/>
       <c r="G79" s="3" t="n"/>
       <c r="H79" s="3" t="n"/>
-      <c r="I79" s="3" t="n"/>
-      <c r="J79" s="3" t="n"/>
-      <c r="K79" s="3" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="3" t="n"/>
@@ -1586,9 +1322,6 @@
       <c r="F80" s="3" t="n"/>
       <c r="G80" s="3" t="n"/>
       <c r="H80" s="3" t="n"/>
-      <c r="I80" s="3" t="n"/>
-      <c r="J80" s="3" t="n"/>
-      <c r="K80" s="3" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="3" t="n"/>
@@ -1599,9 +1332,6 @@
       <c r="F81" s="3" t="n"/>
       <c r="G81" s="3" t="n"/>
       <c r="H81" s="3" t="n"/>
-      <c r="I81" s="3" t="n"/>
-      <c r="J81" s="3" t="n"/>
-      <c r="K81" s="3" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="3" t="n"/>
@@ -1612,9 +1342,6 @@
       <c r="F82" s="3" t="n"/>
       <c r="G82" s="3" t="n"/>
       <c r="H82" s="3" t="n"/>
-      <c r="I82" s="3" t="n"/>
-      <c r="J82" s="3" t="n"/>
-      <c r="K82" s="3" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="3" t="n"/>
@@ -1625,9 +1352,6 @@
       <c r="F83" s="3" t="n"/>
       <c r="G83" s="3" t="n"/>
       <c r="H83" s="3" t="n"/>
-      <c r="I83" s="3" t="n"/>
-      <c r="J83" s="3" t="n"/>
-      <c r="K83" s="3" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="3" t="n"/>
@@ -1638,9 +1362,6 @@
       <c r="F84" s="3" t="n"/>
       <c r="G84" s="3" t="n"/>
       <c r="H84" s="3" t="n"/>
-      <c r="I84" s="3" t="n"/>
-      <c r="J84" s="3" t="n"/>
-      <c r="K84" s="3" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="3" t="n"/>
@@ -1651,9 +1372,6 @@
       <c r="F85" s="3" t="n"/>
       <c r="G85" s="3" t="n"/>
       <c r="H85" s="3" t="n"/>
-      <c r="I85" s="3" t="n"/>
-      <c r="J85" s="3" t="n"/>
-      <c r="K85" s="3" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="3" t="n"/>
@@ -1664,9 +1382,6 @@
       <c r="F86" s="3" t="n"/>
       <c r="G86" s="3" t="n"/>
       <c r="H86" s="3" t="n"/>
-      <c r="I86" s="3" t="n"/>
-      <c r="J86" s="3" t="n"/>
-      <c r="K86" s="3" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="3" t="n"/>
@@ -1677,9 +1392,6 @@
       <c r="F87" s="3" t="n"/>
       <c r="G87" s="3" t="n"/>
       <c r="H87" s="3" t="n"/>
-      <c r="I87" s="3" t="n"/>
-      <c r="J87" s="3" t="n"/>
-      <c r="K87" s="3" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="3" t="n"/>
@@ -1690,9 +1402,6 @@
       <c r="F88" s="3" t="n"/>
       <c r="G88" s="3" t="n"/>
       <c r="H88" s="3" t="n"/>
-      <c r="I88" s="3" t="n"/>
-      <c r="J88" s="3" t="n"/>
-      <c r="K88" s="3" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="3" t="n"/>
@@ -1703,9 +1412,6 @@
       <c r="F89" s="3" t="n"/>
       <c r="G89" s="3" t="n"/>
       <c r="H89" s="3" t="n"/>
-      <c r="I89" s="3" t="n"/>
-      <c r="J89" s="3" t="n"/>
-      <c r="K89" s="3" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="3" t="n"/>
@@ -1716,9 +1422,6 @@
       <c r="F90" s="3" t="n"/>
       <c r="G90" s="3" t="n"/>
       <c r="H90" s="3" t="n"/>
-      <c r="I90" s="3" t="n"/>
-      <c r="J90" s="3" t="n"/>
-      <c r="K90" s="3" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="3" t="n"/>
@@ -1729,9 +1432,6 @@
       <c r="F91" s="3" t="n"/>
       <c r="G91" s="3" t="n"/>
       <c r="H91" s="3" t="n"/>
-      <c r="I91" s="3" t="n"/>
-      <c r="J91" s="3" t="n"/>
-      <c r="K91" s="3" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="3" t="n"/>
@@ -1742,9 +1442,6 @@
       <c r="F92" s="3" t="n"/>
       <c r="G92" s="3" t="n"/>
       <c r="H92" s="3" t="n"/>
-      <c r="I92" s="3" t="n"/>
-      <c r="J92" s="3" t="n"/>
-      <c r="K92" s="3" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="3" t="n"/>
@@ -1755,9 +1452,6 @@
       <c r="F93" s="3" t="n"/>
       <c r="G93" s="3" t="n"/>
       <c r="H93" s="3" t="n"/>
-      <c r="I93" s="3" t="n"/>
-      <c r="J93" s="3" t="n"/>
-      <c r="K93" s="3" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="3" t="n"/>
@@ -1768,9 +1462,6 @@
       <c r="F94" s="3" t="n"/>
       <c r="G94" s="3" t="n"/>
       <c r="H94" s="3" t="n"/>
-      <c r="I94" s="3" t="n"/>
-      <c r="J94" s="3" t="n"/>
-      <c r="K94" s="3" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="3" t="n"/>
@@ -1781,9 +1472,6 @@
       <c r="F95" s="3" t="n"/>
       <c r="G95" s="3" t="n"/>
       <c r="H95" s="3" t="n"/>
-      <c r="I95" s="3" t="n"/>
-      <c r="J95" s="3" t="n"/>
-      <c r="K95" s="3" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="3" t="n"/>
@@ -1794,9 +1482,6 @@
       <c r="F96" s="3" t="n"/>
       <c r="G96" s="3" t="n"/>
       <c r="H96" s="3" t="n"/>
-      <c r="I96" s="3" t="n"/>
-      <c r="J96" s="3" t="n"/>
-      <c r="K96" s="3" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="3" t="n"/>
@@ -1807,9 +1492,6 @@
       <c r="F97" s="3" t="n"/>
       <c r="G97" s="3" t="n"/>
       <c r="H97" s="3" t="n"/>
-      <c r="I97" s="3" t="n"/>
-      <c r="J97" s="3" t="n"/>
-      <c r="K97" s="3" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="3" t="n"/>
@@ -1820,9 +1502,6 @@
       <c r="F98" s="3" t="n"/>
       <c r="G98" s="3" t="n"/>
       <c r="H98" s="3" t="n"/>
-      <c r="I98" s="3" t="n"/>
-      <c r="J98" s="3" t="n"/>
-      <c r="K98" s="3" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="3" t="n"/>
@@ -1833,9 +1512,6 @@
       <c r="F99" s="3" t="n"/>
       <c r="G99" s="3" t="n"/>
       <c r="H99" s="3" t="n"/>
-      <c r="I99" s="3" t="n"/>
-      <c r="J99" s="3" t="n"/>
-      <c r="K99" s="3" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="3" t="n"/>
@@ -1846,9 +1522,6 @@
       <c r="F100" s="3" t="n"/>
       <c r="G100" s="3" t="n"/>
       <c r="H100" s="3" t="n"/>
-      <c r="I100" s="3" t="n"/>
-      <c r="J100" s="3" t="n"/>
-      <c r="K100" s="3" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="3" t="n"/>
@@ -1859,18 +1532,9 @@
       <c r="F101" s="3" t="n"/>
       <c r="G101" s="3" t="n"/>
       <c r="H101" s="3" t="n"/>
-      <c r="I101" s="3" t="n"/>
-      <c r="J101" s="3" t="n"/>
-      <c r="K101" s="3" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="3">
-    <dataValidation sqref="F2:F101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Jefa de marketing,Equipo de marketing,Otra área (solo tickets)"</formula1>
-    </dataValidation>
-    <dataValidation sqref="G2:G101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Sí,No"</formula1>
-    </dataValidation>
+  <dataValidations count="1">
     <dataValidation sqref="E2:E101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Marketing,Comercial,Ventas,Finanzas,Recursos Humanos,Legal,Operaciones,Gerencia,TI,Otra"</formula1>
     </dataValidation>
@@ -1885,7 +1549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1900,7 +1564,7 @@
       </c>
       <c r="B1" s="5" t="inlineStr">
         <is>
-          <t>Una persona por fila en la hoja Personas. Los campos con * son obligatorios. Borra la fila de ejemplo.</t>
+          <t>Una persona por fila en la hoja Personas. Los campos con * son obligatorios. La fila gris es un ejemplo: bórrala.</t>
         </is>
       </c>
     </row>
@@ -1955,72 +1619,46 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Rol en Rabbit</t>
+          <t>Cargo</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Jefa de marketing: aprueba y asigna tickets (solo 1 persona).
-Equipo de marketing: ve Inicio, Mi entorno, Tickets y Dashboard.
-Otra área: solo envía tickets y ve sus solicitudes.</t>
+          <t>Escribe su cargo. Ej.: Diseñadora gráfica, Analista comercial. Con el área definimos qué verá en Rabbit.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>¿Administra Personas?</t>
+          <t>Fecha de cumpleaños</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Sí = puede crear cuentas y restablecer contraseñas (hoy: Hilary y Carlos).</t>
+          <t>Formato día/mes (Ej.: 15/03). Sale en Próximos eventos. Opcional.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Fecha de cumpleaños</t>
+          <t>Celular</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Formato día/mes (Ej.: 15/03). Sale en Próximos eventos. Opcional.</t>
+          <t>Para enviarle por WhatsApp su usuario y contraseña temporal. Opcional.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Celular</t>
+          <t>Contraseña</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Para enviarle por WhatsApp su usuario y contraseña temporal. Opcional.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Foto</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Opcional. Envía las fotos aparte (cuadradas, JPG o PNG) con el nombre que pongas aquí.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Contraseña</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>No la pongas. Rabbit crea una temporal y cada persona elige la suya al entrar la primera vez.</t>
         </is>

</xml_diff>

<commit_message>
Personas: Romano como nombre y usuario
</commit_message>
<xml_diff>
--- a/borradores/rabbit-personas.xlsx
+++ b/borradores/rabbit-personas.xlsx
@@ -863,7 +863,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Cesar</t>
+          <t>Romano</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>cesar</t>
+          <t>romano</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>

</xml_diff>